<commit_message>
Add Harris Teeter data, store-vs-online t-tests, and two-way ANOVA
</commit_message>
<xml_diff>
--- a/data/raw/raw_prices.xlsx
+++ b/data/raw/raw_prices.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="70">
   <si>
     <t>Brand</t>
   </si>
@@ -151,6 +151,15 @@
     <t>Narragansett, 12 pk lager cans</t>
   </si>
   <si>
+    <t>Kind</t>
+  </si>
+  <si>
+    <t>Dark chocolate mocha almond, 12 oz bar</t>
+  </si>
+  <si>
+    <t>Peanut butter dark chocolate, 12 oz bar</t>
+  </si>
+  <si>
     <t>Gazelle</t>
   </si>
   <si>
@@ -172,15 +181,6 @@
     <t>Bulldega</t>
   </si>
   <si>
-    <t>Kind</t>
-  </si>
-  <si>
-    <t>Dark chocolate mocha almond, 12 oz bar</t>
-  </si>
-  <si>
-    <t>Peanut butter dark chocolate, 12 oz bar</t>
-  </si>
-  <si>
     <t xml:space="preserve">Whole Foods Durham </t>
   </si>
   <si>
@@ -218,6 +218,9 @@
   </si>
   <si>
     <t>Almond and sea salt</t>
+  </si>
+  <si>
+    <t>Harris Teeter</t>
   </si>
 </sst>
 </file>
@@ -893,272 +896,272 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>11</v>
+        <v>47</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
       <c r="D29" s="1">
-        <v>2.89</v>
-      </c>
-      <c r="G29" s="1" t="s">
-        <v>47</v>
+        <v>2.29</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
       <c r="D30" s="1">
-        <v>2.89</v>
+        <v>2.29</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>46</v>
+        <v>49</v>
+      </c>
+      <c r="D31" s="1">
+        <v>2.89</v>
+      </c>
+      <c r="G31" s="1" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>46</v>
+        <v>49</v>
+      </c>
+      <c r="D32" s="1">
+        <v>2.89</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="D37" s="1">
-        <v>14.99</v>
-      </c>
-      <c r="G37" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="H37" s="1" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="B39" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D39" s="1">
+        <v>14.99</v>
+      </c>
+      <c r="G39" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C39" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="D39" s="1">
-        <v>2.79</v>
-      </c>
-      <c r="E39" s="1" t="s">
-        <v>30</v>
+      <c r="H39" s="1" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>11</v>
+        <v>45</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="s">
-        <v>26</v>
+        <v>53</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>27</v>
+        <v>54</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>52</v>
+        <v>49</v>
+      </c>
+      <c r="D41" s="1">
+        <v>2.79</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="D42" s="1">
-        <v>3.19</v>
+        <v>55</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="D43" s="1">
-        <v>3.19</v>
+        <v>55</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D44" s="1">
-        <v>2.99</v>
+        <v>3.19</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>52</v>
+        <v>55</v>
+      </c>
+      <c r="D45" s="1">
+        <v>3.19</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>52</v>
+        <v>55</v>
+      </c>
+      <c r="D46" s="1">
+        <v>2.99</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="D47" s="1">
-        <v>17.59</v>
+        <v>55</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="D48" s="1">
-        <v>31.99</v>
+        <v>55</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D49" s="1">
         <v>17.59</v>
@@ -1166,27 +1169,30 @@
     </row>
     <row r="50">
       <c r="A50" s="1" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>52</v>
+        <v>55</v>
+      </c>
+      <c r="D50" s="1">
+        <v>31.99</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D51" s="1">
-        <v>3.99</v>
+        <v>17.59</v>
       </c>
     </row>
     <row r="52">
@@ -1194,83 +1200,86 @@
         <v>53</v>
       </c>
       <c r="B52" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C52" s="1" t="s">
         <v>55</v>
-      </c>
-      <c r="C52" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="D52" s="1">
-        <v>2.99</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>11</v>
+        <v>47</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D53" s="1">
-        <v>2.29</v>
-      </c>
-      <c r="E53" s="1">
-        <v>1.78</v>
-      </c>
-      <c r="F53" s="1" t="s">
-        <v>57</v>
+        <v>3.99</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D54" s="1">
-        <v>2.29</v>
-      </c>
-      <c r="E54" s="1">
-        <v>1.78</v>
-      </c>
-      <c r="F54" s="1" t="s">
-        <v>57</v>
+        <v>2.99</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="C55" s="1" t="s">
         <v>56</v>
       </c>
+      <c r="D55" s="1">
+        <v>2.29</v>
+      </c>
+      <c r="E55" s="1">
+        <v>1.78</v>
+      </c>
+      <c r="F55" s="1" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="C56" s="1" t="s">
         <v>56</v>
       </c>
+      <c r="D56" s="1">
+        <v>2.29</v>
+      </c>
+      <c r="E56" s="1">
+        <v>1.78</v>
+      </c>
+      <c r="F56" s="1" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="C57" s="1" t="s">
         <v>56</v>
@@ -1278,10 +1287,10 @@
     </row>
     <row r="58">
       <c r="A58" s="1" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C58" s="1" t="s">
         <v>56</v>
@@ -1289,95 +1298,83 @@
     </row>
     <row r="59">
       <c r="A59" s="1" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="C59" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D59" s="1">
-        <v>12.99</v>
-      </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C60" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D60" s="1">
-        <v>13.49</v>
-      </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="C61" s="1" t="s">
         <v>56</v>
       </c>
       <c r="D61" s="1">
-        <v>19.49</v>
+        <v>12.99</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C62" s="1" t="s">
         <v>56</v>
       </c>
       <c r="D62" s="1">
-        <v>9.99</v>
-      </c>
-      <c r="F62" s="1" t="s">
-        <v>58</v>
+        <v>13.49</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="C63" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D63" s="1" t="s">
-        <v>59</v>
+      <c r="D63" s="1">
+        <v>19.49</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="C64" s="1" t="s">
         <v>56</v>
       </c>
       <c r="D64" s="1">
-        <v>1.66</v>
-      </c>
-      <c r="E64" s="1">
-        <v>1.49</v>
+        <v>9.99</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="65">
@@ -1385,86 +1382,98 @@
         <v>53</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C65" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D65" s="1">
-        <v>1.66</v>
-      </c>
-      <c r="E65" s="1">
-        <v>1.49</v>
-      </c>
-      <c r="F65" s="1" t="s">
-        <v>61</v>
+      <c r="D65" s="1" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>11</v>
+        <v>47</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="D66" s="1">
-        <v>2.49</v>
+        <v>1.66</v>
       </c>
       <c r="E66" s="1">
-        <v>1.69</v>
+        <v>1.49</v>
+      </c>
+      <c r="F66" s="1" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="D67" s="1">
-        <v>2.19</v>
+        <v>1.66</v>
       </c>
       <c r="E67" s="1">
-        <v>1.69</v>
+        <v>1.49</v>
       </c>
       <c r="F67" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="C68" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="D68" s="1">
+        <v>2.49</v>
+      </c>
+      <c r="E68" s="1">
+        <v>1.69</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="C69" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="D69" s="1">
+        <v>2.19</v>
+      </c>
+      <c r="E69" s="1">
+        <v>1.69</v>
+      </c>
+      <c r="F69" s="1" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="C70" s="1" t="s">
         <v>62</v>
@@ -1472,27 +1481,21 @@
     </row>
     <row r="71">
       <c r="A71" s="1" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C71" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="D71" s="1">
-        <v>1.79</v>
-      </c>
-      <c r="E71" s="1" t="s">
-        <v>64</v>
-      </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="C72" s="1" t="s">
         <v>62</v>
@@ -1500,81 +1503,75 @@
     </row>
     <row r="73">
       <c r="A73" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C73" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="D73" s="1">
+        <v>1.79</v>
+      </c>
+      <c r="E73" s="1" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="C74" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="D74" s="1">
-        <v>20.99</v>
-      </c>
-      <c r="F74" s="1" t="s">
-        <v>9</v>
-      </c>
     </row>
     <row r="75">
       <c r="A75" s="1" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C75" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="D75" s="1">
-        <v>10.49</v>
-      </c>
-      <c r="F75" s="1" t="s">
-        <v>65</v>
-      </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="C76" s="1" t="s">
         <v>62</v>
       </c>
       <c r="D76" s="1">
-        <v>2.59</v>
+        <v>20.99</v>
       </c>
       <c r="F76" s="1" t="s">
-        <v>66</v>
+        <v>9</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="1" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="C77" s="1" t="s">
         <v>62</v>
       </c>
       <c r="D77" s="1">
-        <v>1.79</v>
+        <v>10.49</v>
       </c>
       <c r="F77" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="78">
@@ -1582,16 +1579,217 @@
         <v>53</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C78" s="1" t="s">
         <v>62</v>
       </c>
       <c r="D78" s="1">
+        <v>2.59</v>
+      </c>
+      <c r="F78" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C79" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D79" s="1">
         <v>1.79</v>
       </c>
-      <c r="F78" s="1" t="s">
+      <c r="F79" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C80" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D80" s="1">
+        <v>1.79</v>
+      </c>
+      <c r="F80" s="1" t="s">
         <v>68</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C82" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D82" s="1">
+        <v>2.69</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C83" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D83" s="1">
+        <v>2.69</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C84" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C85" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B86" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C86" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C87" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D87" s="1">
+        <v>2.09</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C88" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B89" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C89" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C90" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D90" s="1">
+        <v>15.99</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C91" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D91" s="1">
+        <v>9.99</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C92" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D92" s="1">
+        <v>2.99</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C93" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D93" s="1">
+        <v>1.99</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C94" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D94" s="1">
+        <v>1.99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>